<commit_message>
Update model outputs 2026-06-26 09:37:45
</commit_message>
<xml_diff>
--- a/files/NRL_anytime_tryscorers.xlsx
+++ b/files/NRL_anytime_tryscorers.xlsx
@@ -1266,7 +1266,7 @@
         <v>1</v>
       </c>
       <c r="I2" s="4" t="n">
-        <v>2.22</v>
+        <v>2.19</v>
       </c>
     </row>
     <row r="3">
@@ -1295,7 +1295,7 @@
         <v>1</v>
       </c>
       <c r="I3" s="4" t="n">
-        <v>2.66</v>
+        <v>2.62</v>
       </c>
     </row>
     <row r="4">
@@ -1324,7 +1324,7 @@
         <v>1</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>3.35</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="5">
@@ -1353,7 +1353,7 @@
         <v>1</v>
       </c>
       <c r="I5" s="4" t="n">
-        <v>3.7</v>
+        <v>3.64</v>
       </c>
     </row>
     <row r="6">
@@ -1382,7 +1382,7 @@
         <v>1</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>4.27</v>
+        <v>4.21</v>
       </c>
     </row>
     <row r="7">
@@ -1411,7 +1411,7 @@
         <v>1</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>4.66</v>
+        <v>4.58</v>
       </c>
     </row>
     <row r="8">
@@ -1440,7 +1440,7 @@
         <v>1</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>4.66</v>
+        <v>4.58</v>
       </c>
     </row>
     <row r="9">
@@ -1469,7 +1469,7 @@
         <v>1</v>
       </c>
       <c r="I9" s="4" t="n">
-        <v>4.72</v>
+        <v>4.65</v>
       </c>
     </row>
     <row r="10">
@@ -1498,7 +1498,7 @@
         <v>1</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>4.99</v>
+        <v>4.91</v>
       </c>
     </row>
     <row r="11">
@@ -1527,7 +1527,7 @@
         <v>1</v>
       </c>
       <c r="I11" s="4" t="n">
-        <v>5.3</v>
+        <v>5.21</v>
       </c>
     </row>
     <row r="12">
@@ -1556,7 +1556,7 @@
         <v>0</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>8.32</v>
+        <v>8.18</v>
       </c>
     </row>
     <row r="13">
@@ -1585,7 +1585,7 @@
         <v>1</v>
       </c>
       <c r="I13" s="4" t="n">
-        <v>11.07</v>
+        <v>10.88</v>
       </c>
     </row>
     <row r="14">
@@ -1614,7 +1614,7 @@
         <v>1</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>13.93</v>
+        <v>13.68</v>
       </c>
     </row>
     <row r="15">
@@ -1643,7 +1643,7 @@
         <v>1</v>
       </c>
       <c r="I15" s="4" t="n">
-        <v>14.16</v>
+        <v>13.91</v>
       </c>
     </row>
     <row r="16">
@@ -1672,7 +1672,7 @@
         <v>1</v>
       </c>
       <c r="I16" s="4" t="n">
-        <v>1.78</v>
+        <v>1.76</v>
       </c>
     </row>
     <row r="17">
@@ -1701,7 +1701,7 @@
         <v>1</v>
       </c>
       <c r="I17" s="4" t="n">
-        <v>2.73</v>
+        <v>2.68</v>
       </c>
     </row>
     <row r="18">
@@ -1730,7 +1730,7 @@
         <v>1</v>
       </c>
       <c r="I18" s="4" t="n">
-        <v>3.33</v>
+        <v>3.26</v>
       </c>
     </row>
     <row r="19">
@@ -1759,7 +1759,7 @@
         <v>1</v>
       </c>
       <c r="I19" s="4" t="n">
-        <v>3.37</v>
+        <v>3.31</v>
       </c>
     </row>
     <row r="20">
@@ -1788,7 +1788,7 @@
         <v>1</v>
       </c>
       <c r="I20" s="4" t="n">
-        <v>3.7</v>
+        <v>3.63</v>
       </c>
     </row>
     <row r="21">
@@ -1817,7 +1817,7 @@
         <v>1</v>
       </c>
       <c r="I21" s="4" t="n">
-        <v>4.74</v>
+        <v>4.64</v>
       </c>
     </row>
     <row r="22">
@@ -1846,7 +1846,7 @@
         <v>1</v>
       </c>
       <c r="I22" s="4" t="n">
-        <v>4.74</v>
+        <v>4.64</v>
       </c>
     </row>
     <row r="23">
@@ -1875,7 +1875,7 @@
         <v>1</v>
       </c>
       <c r="I23" s="4" t="n">
-        <v>5.14</v>
+        <v>5.04</v>
       </c>
     </row>
     <row r="24">
@@ -1904,7 +1904,7 @@
         <v>1</v>
       </c>
       <c r="I24" s="4" t="n">
-        <v>7.09</v>
+        <v>6.94</v>
       </c>
     </row>
     <row r="25">
@@ -1933,7 +1933,7 @@
         <v>1</v>
       </c>
       <c r="I25" s="4" t="n">
-        <v>7.6</v>
+        <v>7.43</v>
       </c>
     </row>
     <row r="26">
@@ -1962,7 +1962,7 @@
         <v>1</v>
       </c>
       <c r="I26" s="4" t="n">
-        <v>7.99</v>
+        <v>7.82</v>
       </c>
     </row>
     <row r="27">
@@ -1991,7 +1991,7 @@
         <v>0</v>
       </c>
       <c r="I27" s="4" t="n">
-        <v>9.63</v>
+        <v>9.42</v>
       </c>
     </row>
     <row r="28">
@@ -2020,7 +2020,7 @@
         <v>0</v>
       </c>
       <c r="I28" s="4" t="n">
-        <v>10.18</v>
+        <v>9.96</v>
       </c>
     </row>
     <row r="29">
@@ -2049,7 +2049,7 @@
         <v>1</v>
       </c>
       <c r="I29" s="4" t="n">
-        <v>11.01</v>
+        <v>10.77</v>
       </c>
     </row>
     <row r="30">
@@ -2078,7 +2078,7 @@
         <v>0</v>
       </c>
       <c r="I30" s="4" t="n">
-        <v>12.43</v>
+        <v>12.16</v>
       </c>
     </row>
     <row r="31">
@@ -2107,7 +2107,7 @@
         <v>1</v>
       </c>
       <c r="I31" s="4" t="n">
-        <v>13.66</v>
+        <v>13.36</v>
       </c>
     </row>
     <row r="32">

</xml_diff>